<commit_message>
Prompt caching: the fixed instructions are cached for an hour, the changing part (time, Shabbat, this customer) comes after; demo shows the cost per message; AI cost in the expenses sheet updated to about 11 USD a month
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASRMwiCmV7VLN1LwrbbDK1
</commit_message>
<xml_diff>
--- a/automation-agency/expenses.xlsx
+++ b/automation-agency/expenses.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="93">
   <si>
     <t xml:space="preserve">סיכום: עונה ראשון</t>
   </si>
@@ -283,7 +283,10 @@
     <t xml:space="preserve">לכל לקוח</t>
   </si>
   <si>
-    <t xml:space="preserve">הערכה ללקוח עם כ-90 פניות בחודש. גדל עם מספר הפניות</t>
+    <t xml:space="preserve">15/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">הערכה ללקוח עם כ-85 פניות בחודש, עם "זיכרון זמני" (בלי זה: כ-20 דולר). לעדכן אחרי שבוע אמיתי</t>
   </si>
   <si>
     <t xml:space="preserve">360dialog, חיבור רשמי למספר של הלקוח</t>
@@ -489,36 +492,40 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -538,11 +545,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -558,7 +565,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -876,135 +883,135 @@
   <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="56"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <f aca="false">SUMIFS(הוצאות!$L$5:$L$31,הוצאות!$G$5:$G$31,"קבוע",הוצאות!$F$5:$F$31,"&lt;&gt;בוטל")</f>
         <v>162.8</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <f aca="false">SUMIFS(הוצאות!$L$5:$L$31,הוצאות!$G$5:$G$31,"לכל לקוח",הוצאות!$F$5:$F$31,"&lt;&gt;בוטל")</f>
-        <v>261.5</v>
-      </c>
-      <c r="C6" s="2" t="s">
+        <v>246.7</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <f aca="false">הגדרות!$B$6</f>
         <v>500</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <f aca="false">SUMIFS(הוצאות!$L$5:$L$31,הוצאות!$F$5:$F$31,"פעיל")</f>
-        <v>218.3</v>
-      </c>
-      <c r="C10" s="2" t="s">
+        <v>203.5</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <f aca="false">B9-B10</f>
-        <v>281.7</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+        <v>296.5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="8" t="n">
         <f aca="false">B9-B5-B6</f>
-        <v>75.7</v>
-      </c>
-      <c r="C12" s="2" t="s">
+        <v>90.5</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="6" t="n">
         <f aca="false">SUMIFS(הוצאות!$K$5:$K$31,הוצאות!$E$5:$E$31,"חד-פעמי",הוצאות!$F$5:$F$31,"פעיל")</f>
         <v>37</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="6" t="n">
         <f aca="false">הגדרות!$B$8</f>
         <v>2500</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="6" t="n">
         <f aca="false">הגדרות!$B$8-הגדרות!$B$9</f>
         <v>1500</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1027,797 +1034,797 @@
   <dimension ref="A1:I26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="28"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A5-1)*הגדרות!$B$7</f>
         <v>500</v>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="11" t="n">
         <f aca="false">A5*סיכום!$B$6</f>
-        <v>261.5</v>
-      </c>
-      <c r="E5" s="11" t="n">
+        <v>246.7</v>
+      </c>
+      <c r="E5" s="12" t="n">
         <f aca="false">B5-C5-D5</f>
-        <v>75.7</v>
-      </c>
-      <c r="F5" s="10" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="F5" s="11" t="n">
         <f aca="false">E5/A5</f>
-        <v>75.7</v>
-      </c>
-      <c r="G5" s="10" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="G5" s="11" t="n">
         <f aca="false">E5*12</f>
-        <v>908.4</v>
-      </c>
-      <c r="H5" s="10" t="n">
+        <v>1086</v>
+      </c>
+      <c r="H5" s="11" t="n">
         <f aca="false">B5*12</f>
         <v>6000</v>
       </c>
-      <c r="I5" s="10" t="str">
+      <c r="I5" s="11" t="str">
         <f aca="false">IF(H5&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A6-1)*הגדרות!$B$7</f>
         <v>1090</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="11" t="n">
         <f aca="false">A6*סיכום!$B$6</f>
-        <v>523</v>
-      </c>
-      <c r="E6" s="11" t="n">
+        <v>493.4</v>
+      </c>
+      <c r="E6" s="12" t="n">
         <f aca="false">B6-C6-D6</f>
-        <v>404.2</v>
-      </c>
-      <c r="F6" s="10" t="n">
+        <v>433.8</v>
+      </c>
+      <c r="F6" s="11" t="n">
         <f aca="false">E6/A6</f>
-        <v>202.1</v>
-      </c>
-      <c r="G6" s="10" t="n">
+        <v>216.9</v>
+      </c>
+      <c r="G6" s="11" t="n">
         <f aca="false">E6*12</f>
-        <v>4850.4</v>
-      </c>
-      <c r="H6" s="10" t="n">
+        <v>5205.6</v>
+      </c>
+      <c r="H6" s="11" t="n">
         <f aca="false">B6*12</f>
         <v>13080</v>
       </c>
-      <c r="I6" s="10" t="str">
+      <c r="I6" s="11" t="str">
         <f aca="false">IF(H6&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A7-1)*הגדרות!$B$7</f>
         <v>1680</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <f aca="false">A7*סיכום!$B$6</f>
-        <v>784.5</v>
-      </c>
-      <c r="E7" s="11" t="n">
+        <v>740.1</v>
+      </c>
+      <c r="E7" s="12" t="n">
         <f aca="false">B7-C7-D7</f>
-        <v>732.7</v>
-      </c>
-      <c r="F7" s="10" t="n">
+        <v>777.1</v>
+      </c>
+      <c r="F7" s="11" t="n">
         <f aca="false">E7/A7</f>
-        <v>244.233333333333</v>
-      </c>
-      <c r="G7" s="10" t="n">
+        <v>259.033333333333</v>
+      </c>
+      <c r="G7" s="11" t="n">
         <f aca="false">E7*12</f>
-        <v>8792.4</v>
-      </c>
-      <c r="H7" s="10" t="n">
+        <v>9325.2</v>
+      </c>
+      <c r="H7" s="11" t="n">
         <f aca="false">B7*12</f>
         <v>20160</v>
       </c>
-      <c r="I7" s="10" t="str">
+      <c r="I7" s="11" t="str">
         <f aca="false">IF(H7&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A8-1)*הגדרות!$B$7</f>
         <v>2270</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="11" t="n">
         <f aca="false">A8*סיכום!$B$6</f>
-        <v>1046</v>
-      </c>
-      <c r="E8" s="11" t="n">
+        <v>986.8</v>
+      </c>
+      <c r="E8" s="12" t="n">
         <f aca="false">B8-C8-D8</f>
-        <v>1061.2</v>
-      </c>
-      <c r="F8" s="10" t="n">
+        <v>1120.4</v>
+      </c>
+      <c r="F8" s="11" t="n">
         <f aca="false">E8/A8</f>
-        <v>265.3</v>
-      </c>
-      <c r="G8" s="10" t="n">
+        <v>280.1</v>
+      </c>
+      <c r="G8" s="11" t="n">
         <f aca="false">E8*12</f>
-        <v>12734.4</v>
-      </c>
-      <c r="H8" s="10" t="n">
+        <v>13444.8</v>
+      </c>
+      <c r="H8" s="11" t="n">
         <f aca="false">B8*12</f>
         <v>27240</v>
       </c>
-      <c r="I8" s="10" t="str">
+      <c r="I8" s="11" t="str">
         <f aca="false">IF(H8&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A9-1)*הגדרות!$B$7</f>
         <v>2860</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="11" t="n">
         <f aca="false">A9*סיכום!$B$6</f>
-        <v>1307.5</v>
-      </c>
-      <c r="E9" s="11" t="n">
+        <v>1233.5</v>
+      </c>
+      <c r="E9" s="12" t="n">
         <f aca="false">B9-C9-D9</f>
-        <v>1389.7</v>
-      </c>
-      <c r="F9" s="10" t="n">
+        <v>1463.7</v>
+      </c>
+      <c r="F9" s="11" t="n">
         <f aca="false">E9/A9</f>
-        <v>277.94</v>
-      </c>
-      <c r="G9" s="10" t="n">
+        <v>292.74</v>
+      </c>
+      <c r="G9" s="11" t="n">
         <f aca="false">E9*12</f>
-        <v>16676.4</v>
-      </c>
-      <c r="H9" s="10" t="n">
+        <v>17564.4</v>
+      </c>
+      <c r="H9" s="11" t="n">
         <f aca="false">B9*12</f>
         <v>34320</v>
       </c>
-      <c r="I9" s="10" t="str">
+      <c r="I9" s="11" t="str">
         <f aca="false">IF(H9&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A10-1)*הגדרות!$B$7</f>
         <v>3450</v>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="11" t="n">
         <f aca="false">A10*סיכום!$B$6</f>
-        <v>1569</v>
-      </c>
-      <c r="E10" s="11" t="n">
+        <v>1480.2</v>
+      </c>
+      <c r="E10" s="12" t="n">
         <f aca="false">B10-C10-D10</f>
-        <v>1718.2</v>
-      </c>
-      <c r="F10" s="10" t="n">
+        <v>1807</v>
+      </c>
+      <c r="F10" s="11" t="n">
         <f aca="false">E10/A10</f>
-        <v>286.366666666667</v>
-      </c>
-      <c r="G10" s="10" t="n">
+        <v>301.166666666667</v>
+      </c>
+      <c r="G10" s="11" t="n">
         <f aca="false">E10*12</f>
-        <v>20618.4</v>
-      </c>
-      <c r="H10" s="10" t="n">
+        <v>21684</v>
+      </c>
+      <c r="H10" s="11" t="n">
         <f aca="false">B10*12</f>
         <v>41400</v>
       </c>
-      <c r="I10" s="10" t="str">
+      <c r="I10" s="11" t="str">
         <f aca="false">IF(H10&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A11-1)*הגדרות!$B$7</f>
         <v>4040</v>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="11" t="n">
         <f aca="false">A11*סיכום!$B$6</f>
-        <v>1830.5</v>
-      </c>
-      <c r="E11" s="11" t="n">
+        <v>1726.9</v>
+      </c>
+      <c r="E11" s="12" t="n">
         <f aca="false">B11-C11-D11</f>
-        <v>2046.7</v>
-      </c>
-      <c r="F11" s="10" t="n">
+        <v>2150.3</v>
+      </c>
+      <c r="F11" s="11" t="n">
         <f aca="false">E11/A11</f>
-        <v>292.385714285714</v>
-      </c>
-      <c r="G11" s="10" t="n">
+        <v>307.185714285714</v>
+      </c>
+      <c r="G11" s="11" t="n">
         <f aca="false">E11*12</f>
-        <v>24560.4</v>
-      </c>
-      <c r="H11" s="10" t="n">
+        <v>25803.6</v>
+      </c>
+      <c r="H11" s="11" t="n">
         <f aca="false">B11*12</f>
         <v>48480</v>
       </c>
-      <c r="I11" s="10" t="str">
+      <c r="I11" s="11" t="str">
         <f aca="false">IF(H11&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A12-1)*הגדרות!$B$7</f>
         <v>4630</v>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D12" s="11" t="n">
         <f aca="false">A12*סיכום!$B$6</f>
-        <v>2092</v>
-      </c>
-      <c r="E12" s="11" t="n">
+        <v>1973.6</v>
+      </c>
+      <c r="E12" s="12" t="n">
         <f aca="false">B12-C12-D12</f>
-        <v>2375.2</v>
-      </c>
-      <c r="F12" s="10" t="n">
+        <v>2493.6</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <f aca="false">E12/A12</f>
-        <v>296.9</v>
-      </c>
-      <c r="G12" s="10" t="n">
+        <v>311.7</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <f aca="false">E12*12</f>
-        <v>28502.4</v>
-      </c>
-      <c r="H12" s="10" t="n">
+        <v>29923.2</v>
+      </c>
+      <c r="H12" s="11" t="n">
         <f aca="false">B12*12</f>
         <v>55560</v>
       </c>
-      <c r="I12" s="10" t="str">
+      <c r="I12" s="11" t="str">
         <f aca="false">IF(H12&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A13-1)*הגדרות!$B$7</f>
         <v>5220</v>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="11" t="n">
         <f aca="false">A13*סיכום!$B$6</f>
-        <v>2353.5</v>
-      </c>
-      <c r="E13" s="11" t="n">
+        <v>2220.3</v>
+      </c>
+      <c r="E13" s="12" t="n">
         <f aca="false">B13-C13-D13</f>
-        <v>2703.7</v>
-      </c>
-      <c r="F13" s="10" t="n">
+        <v>2836.9</v>
+      </c>
+      <c r="F13" s="11" t="n">
         <f aca="false">E13/A13</f>
-        <v>300.411111111111</v>
-      </c>
-      <c r="G13" s="10" t="n">
+        <v>315.211111111111</v>
+      </c>
+      <c r="G13" s="11" t="n">
         <f aca="false">E13*12</f>
-        <v>32444.4</v>
-      </c>
-      <c r="H13" s="10" t="n">
+        <v>34042.8</v>
+      </c>
+      <c r="H13" s="11" t="n">
         <f aca="false">B13*12</f>
         <v>62640</v>
       </c>
-      <c r="I13" s="10" t="str">
+      <c r="I13" s="11" t="str">
         <f aca="false">IF(H13&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A14-1)*הגדרות!$B$7</f>
         <v>5810</v>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="11" t="n">
         <f aca="false">A14*סיכום!$B$6</f>
-        <v>2615</v>
-      </c>
-      <c r="E14" s="11" t="n">
+        <v>2467</v>
+      </c>
+      <c r="E14" s="12" t="n">
         <f aca="false">B14-C14-D14</f>
-        <v>3032.2</v>
-      </c>
-      <c r="F14" s="10" t="n">
+        <v>3180.2</v>
+      </c>
+      <c r="F14" s="11" t="n">
         <f aca="false">E14/A14</f>
-        <v>303.22</v>
-      </c>
-      <c r="G14" s="10" t="n">
+        <v>318.02</v>
+      </c>
+      <c r="G14" s="11" t="n">
         <f aca="false">E14*12</f>
-        <v>36386.4</v>
-      </c>
-      <c r="H14" s="10" t="n">
+        <v>38162.4</v>
+      </c>
+      <c r="H14" s="11" t="n">
         <f aca="false">B14*12</f>
         <v>69720</v>
       </c>
-      <c r="I14" s="10" t="str">
+      <c r="I14" s="11" t="str">
         <f aca="false">IF(H14&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A15-1)*הגדרות!$B$7</f>
         <v>6400</v>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="11" t="n">
         <f aca="false">A15*סיכום!$B$6</f>
-        <v>2876.5</v>
-      </c>
-      <c r="E15" s="11" t="n">
+        <v>2713.7</v>
+      </c>
+      <c r="E15" s="12" t="n">
         <f aca="false">B15-C15-D15</f>
-        <v>3360.7</v>
-      </c>
-      <c r="F15" s="10" t="n">
+        <v>3523.5</v>
+      </c>
+      <c r="F15" s="11" t="n">
         <f aca="false">E15/A15</f>
-        <v>305.518181818182</v>
-      </c>
-      <c r="G15" s="10" t="n">
+        <v>320.318181818182</v>
+      </c>
+      <c r="G15" s="11" t="n">
         <f aca="false">E15*12</f>
-        <v>40328.4</v>
-      </c>
-      <c r="H15" s="10" t="n">
+        <v>42282</v>
+      </c>
+      <c r="H15" s="11" t="n">
         <f aca="false">B15*12</f>
         <v>76800</v>
       </c>
-      <c r="I15" s="10" t="str">
+      <c r="I15" s="11" t="str">
         <f aca="false">IF(H15&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A16-1)*הגדרות!$B$7</f>
         <v>6990</v>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C16" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D16" s="11" t="n">
         <f aca="false">A16*סיכום!$B$6</f>
-        <v>3138</v>
-      </c>
-      <c r="E16" s="11" t="n">
+        <v>2960.4</v>
+      </c>
+      <c r="E16" s="12" t="n">
         <f aca="false">B16-C16-D16</f>
-        <v>3689.2</v>
-      </c>
-      <c r="F16" s="10" t="n">
+        <v>3866.8</v>
+      </c>
+      <c r="F16" s="11" t="n">
         <f aca="false">E16/A16</f>
-        <v>307.433333333333</v>
-      </c>
-      <c r="G16" s="10" t="n">
+        <v>322.233333333333</v>
+      </c>
+      <c r="G16" s="11" t="n">
         <f aca="false">E16*12</f>
-        <v>44270.4</v>
-      </c>
-      <c r="H16" s="10" t="n">
+        <v>46401.6</v>
+      </c>
+      <c r="H16" s="11" t="n">
         <f aca="false">B16*12</f>
         <v>83880</v>
       </c>
-      <c r="I16" s="10" t="str">
+      <c r="I16" s="11" t="str">
         <f aca="false">IF(H16&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A17-1)*הגדרות!$B$7</f>
         <v>7580</v>
       </c>
-      <c r="C17" s="10" t="n">
+      <c r="C17" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D17" s="11" t="n">
         <f aca="false">A17*סיכום!$B$6</f>
-        <v>3399.5</v>
-      </c>
-      <c r="E17" s="11" t="n">
+        <v>3207.1</v>
+      </c>
+      <c r="E17" s="12" t="n">
         <f aca="false">B17-C17-D17</f>
-        <v>4017.7</v>
-      </c>
-      <c r="F17" s="10" t="n">
+        <v>4210.1</v>
+      </c>
+      <c r="F17" s="11" t="n">
         <f aca="false">E17/A17</f>
-        <v>309.053846153846</v>
-      </c>
-      <c r="G17" s="10" t="n">
+        <v>323.853846153846</v>
+      </c>
+      <c r="G17" s="11" t="n">
         <f aca="false">E17*12</f>
-        <v>48212.4</v>
-      </c>
-      <c r="H17" s="10" t="n">
+        <v>50521.2</v>
+      </c>
+      <c r="H17" s="11" t="n">
         <f aca="false">B17*12</f>
         <v>90960</v>
       </c>
-      <c r="I17" s="10" t="str">
+      <c r="I17" s="11" t="str">
         <f aca="false">IF(H17&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A18-1)*הגדרות!$B$7</f>
         <v>8170</v>
       </c>
-      <c r="C18" s="10" t="n">
+      <c r="C18" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D18" s="11" t="n">
         <f aca="false">A18*סיכום!$B$6</f>
-        <v>3661</v>
-      </c>
-      <c r="E18" s="11" t="n">
+        <v>3453.8</v>
+      </c>
+      <c r="E18" s="12" t="n">
         <f aca="false">B18-C18-D18</f>
-        <v>4346.2</v>
-      </c>
-      <c r="F18" s="10" t="n">
+        <v>4553.4</v>
+      </c>
+      <c r="F18" s="11" t="n">
         <f aca="false">E18/A18</f>
-        <v>310.442857142857</v>
-      </c>
-      <c r="G18" s="10" t="n">
+        <v>325.242857142857</v>
+      </c>
+      <c r="G18" s="11" t="n">
         <f aca="false">E18*12</f>
-        <v>52154.4</v>
-      </c>
-      <c r="H18" s="10" t="n">
+        <v>54640.8</v>
+      </c>
+      <c r="H18" s="11" t="n">
         <f aca="false">B18*12</f>
         <v>98040</v>
       </c>
-      <c r="I18" s="10" t="str">
+      <c r="I18" s="11" t="str">
         <f aca="false">IF(H18&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A19-1)*הגדרות!$B$7</f>
         <v>8760</v>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="11" t="n">
         <f aca="false">A19*סיכום!$B$6</f>
-        <v>3922.5</v>
-      </c>
-      <c r="E19" s="11" t="n">
+        <v>3700.5</v>
+      </c>
+      <c r="E19" s="12" t="n">
         <f aca="false">B19-C19-D19</f>
-        <v>4674.7</v>
-      </c>
-      <c r="F19" s="10" t="n">
+        <v>4896.7</v>
+      </c>
+      <c r="F19" s="11" t="n">
         <f aca="false">E19/A19</f>
-        <v>311.646666666667</v>
-      </c>
-      <c r="G19" s="10" t="n">
+        <v>326.446666666667</v>
+      </c>
+      <c r="G19" s="11" t="n">
         <f aca="false">E19*12</f>
-        <v>56096.4</v>
-      </c>
-      <c r="H19" s="10" t="n">
+        <v>58760.4</v>
+      </c>
+      <c r="H19" s="11" t="n">
         <f aca="false">B19*12</f>
         <v>105120</v>
       </c>
-      <c r="I19" s="10" t="str">
+      <c r="I19" s="11" t="str">
         <f aca="false">IF(H19&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A20-1)*הגדרות!$B$7</f>
         <v>9350</v>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="D20" s="11" t="n">
         <f aca="false">A20*סיכום!$B$6</f>
-        <v>4184</v>
-      </c>
-      <c r="E20" s="11" t="n">
+        <v>3947.2</v>
+      </c>
+      <c r="E20" s="12" t="n">
         <f aca="false">B20-C20-D20</f>
-        <v>5003.2</v>
-      </c>
-      <c r="F20" s="10" t="n">
+        <v>5240</v>
+      </c>
+      <c r="F20" s="11" t="n">
         <f aca="false">E20/A20</f>
-        <v>312.7</v>
-      </c>
-      <c r="G20" s="10" t="n">
+        <v>327.5</v>
+      </c>
+      <c r="G20" s="11" t="n">
         <f aca="false">E20*12</f>
-        <v>60038.4</v>
-      </c>
-      <c r="H20" s="10" t="n">
+        <v>62880</v>
+      </c>
+      <c r="H20" s="11" t="n">
         <f aca="false">B20*12</f>
         <v>112200</v>
       </c>
-      <c r="I20" s="10" t="str">
+      <c r="I20" s="11" t="str">
         <f aca="false">IF(H20&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A21-1)*הגדרות!$B$7</f>
         <v>9940</v>
       </c>
-      <c r="C21" s="10" t="n">
+      <c r="C21" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="11" t="n">
         <f aca="false">A21*סיכום!$B$6</f>
-        <v>4445.5</v>
-      </c>
-      <c r="E21" s="11" t="n">
+        <v>4193.9</v>
+      </c>
+      <c r="E21" s="12" t="n">
         <f aca="false">B21-C21-D21</f>
-        <v>5331.7</v>
-      </c>
-      <c r="F21" s="10" t="n">
+        <v>5583.3</v>
+      </c>
+      <c r="F21" s="11" t="n">
         <f aca="false">E21/A21</f>
-        <v>313.629411764706</v>
-      </c>
-      <c r="G21" s="10" t="n">
+        <v>328.429411764706</v>
+      </c>
+      <c r="G21" s="11" t="n">
         <f aca="false">E21*12</f>
-        <v>63980.4</v>
-      </c>
-      <c r="H21" s="10" t="n">
+        <v>66999.6</v>
+      </c>
+      <c r="H21" s="11" t="n">
         <f aca="false">B21*12</f>
         <v>119280</v>
       </c>
-      <c r="I21" s="10" t="str">
+      <c r="I21" s="11" t="str">
         <f aca="false">IF(H21&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>לא</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="10" t="n">
+      <c r="B22" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A22-1)*הגדרות!$B$7</f>
         <v>10530</v>
       </c>
-      <c r="C22" s="10" t="n">
+      <c r="C22" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D22" s="10" t="n">
+      <c r="D22" s="11" t="n">
         <f aca="false">A22*סיכום!$B$6</f>
-        <v>4707</v>
-      </c>
-      <c r="E22" s="11" t="n">
+        <v>4440.6</v>
+      </c>
+      <c r="E22" s="12" t="n">
         <f aca="false">B22-C22-D22</f>
-        <v>5660.2</v>
-      </c>
-      <c r="F22" s="10" t="n">
+        <v>5926.6</v>
+      </c>
+      <c r="F22" s="11" t="n">
         <f aca="false">E22/A22</f>
-        <v>314.455555555556</v>
-      </c>
-      <c r="G22" s="10" t="n">
+        <v>329.255555555556</v>
+      </c>
+      <c r="G22" s="11" t="n">
         <f aca="false">E22*12</f>
-        <v>67922.4</v>
-      </c>
-      <c r="H22" s="10" t="n">
+        <v>71119.2</v>
+      </c>
+      <c r="H22" s="11" t="n">
         <f aca="false">B22*12</f>
         <v>126360</v>
       </c>
-      <c r="I22" s="10" t="str">
+      <c r="I22" s="11" t="str">
         <f aca="false">IF(H22&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>כן, צריך לעבור לעוסק מורשה</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="10" t="n">
+      <c r="B23" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A23-1)*הגדרות!$B$7</f>
         <v>11120</v>
       </c>
-      <c r="C23" s="10" t="n">
+      <c r="C23" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D23" s="10" t="n">
+      <c r="D23" s="11" t="n">
         <f aca="false">A23*סיכום!$B$6</f>
-        <v>4968.5</v>
-      </c>
-      <c r="E23" s="11" t="n">
+        <v>4687.3</v>
+      </c>
+      <c r="E23" s="12" t="n">
         <f aca="false">B23-C23-D23</f>
-        <v>5988.7</v>
-      </c>
-      <c r="F23" s="10" t="n">
+        <v>6269.9</v>
+      </c>
+      <c r="F23" s="11" t="n">
         <f aca="false">E23/A23</f>
-        <v>315.194736842105</v>
-      </c>
-      <c r="G23" s="10" t="n">
+        <v>329.994736842105</v>
+      </c>
+      <c r="G23" s="11" t="n">
         <f aca="false">E23*12</f>
-        <v>71864.4</v>
-      </c>
-      <c r="H23" s="10" t="n">
+        <v>75238.8</v>
+      </c>
+      <c r="H23" s="11" t="n">
         <f aca="false">B23*12</f>
         <v>133440</v>
       </c>
-      <c r="I23" s="10" t="str">
+      <c r="I23" s="11" t="str">
         <f aca="false">IF(H23&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>כן, צריך לעבור לעוסק מורשה</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="10" t="n">
+      <c r="B24" s="11" t="n">
         <f aca="false">הגדרות!$B$6+(A24-1)*הגדרות!$B$7</f>
         <v>11710</v>
       </c>
-      <c r="C24" s="10" t="n">
+      <c r="C24" s="11" t="n">
         <f aca="false">סיכום!$B$5</f>
         <v>162.8</v>
       </c>
-      <c r="D24" s="10" t="n">
+      <c r="D24" s="11" t="n">
         <f aca="false">A24*סיכום!$B$6</f>
-        <v>5230</v>
-      </c>
-      <c r="E24" s="11" t="n">
+        <v>4934</v>
+      </c>
+      <c r="E24" s="12" t="n">
         <f aca="false">B24-C24-D24</f>
-        <v>6317.2</v>
-      </c>
-      <c r="F24" s="10" t="n">
+        <v>6613.2</v>
+      </c>
+      <c r="F24" s="11" t="n">
         <f aca="false">E24/A24</f>
-        <v>315.86</v>
-      </c>
-      <c r="G24" s="10" t="n">
+        <v>330.66</v>
+      </c>
+      <c r="G24" s="11" t="n">
         <f aca="false">E24*12</f>
-        <v>75806.4</v>
-      </c>
-      <c r="H24" s="10" t="n">
+        <v>79358.4</v>
+      </c>
+      <c r="H24" s="11" t="n">
         <f aca="false">B24*12</f>
         <v>140520</v>
       </c>
-      <c r="I24" s="10" t="str">
+      <c r="I24" s="11" t="str">
         <f aca="false">IF(H24&gt;הגדרות!$B$10,"כן, צריך לעבור לעוסק מורשה","לא")</f>
         <v>כן, צריך לעבור לעוסק מורשה</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1845,95 +1852,95 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="13" t="n">
         <v>3.7</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="14" t="n">
         <v>500</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="14" t="n">
         <v>590</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="14" t="n">
         <v>2500</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="14" t="n">
         <v>1000</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="14" t="n">
         <v>120000</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1956,737 +1963,737 @@
   <dimension ref="A1:L31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="H5" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="I5" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="J5" s="14" t="s">
+      <c r="J5" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="K5" s="17" t="n">
+      <c r="K5" s="18" t="n">
         <f aca="false">IF(C5="","",C5*IF(D5="USD",הגדרות!$B$4,IF(D5="EUR",הגדרות!$B$5,1)))</f>
         <v>18.5</v>
       </c>
-      <c r="L5" s="17" t="n">
+      <c r="L5" s="18" t="n">
         <f aca="false">IF(C5="","",IF(OR(E5="חודשי",E5="לפי שימוש"),K5,IF(E5="שנתי",K5/12,0)))</f>
         <v>18.5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
+    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="17" t="n">
         <v>39</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="H6" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="I6" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="J6" s="14" t="s">
+      <c r="J6" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="K6" s="17" t="n">
+      <c r="K6" s="18" t="n">
         <f aca="false">IF(C6="","",C6*IF(D6="USD",הגדרות!$B$4,IF(D6="EUR",הגדרות!$B$5,1)))</f>
         <v>144.3</v>
       </c>
-      <c r="L6" s="17" t="n">
+      <c r="L6" s="18" t="n">
         <f aca="false">IF(C6="","",IF(OR(E6="חודשי",E6="לפי שימוש"),K6,IF(E6="שנתי",K6/12,0)))</f>
         <v>144.3</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="G7" s="15" t="s">
+      <c r="G7" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="H7" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="I7" s="15" t="s">
+      <c r="I7" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="J7" s="14" t="s">
+      <c r="J7" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="K7" s="17" t="n">
+      <c r="K7" s="18" t="n">
         <f aca="false">IF(C7="","",C7*IF(D7="USD",הגדרות!$B$4,IF(D7="EUR",הגדרות!$B$5,1)))</f>
         <v>0</v>
       </c>
-      <c r="L7" s="17" t="n">
+      <c r="L7" s="18" t="n">
         <f aca="false">IF(C7="","",IF(OR(E7="חודשי",E7="לפי שימוש"),K7,IF(E7="שנתי",K7/12,0)))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="G8" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="H8" s="15" t="s">
+      <c r="H8" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J8" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="K8" s="17" t="n">
+      <c r="K8" s="18" t="n">
         <f aca="false">IF(C8="","",C8*IF(D8="USD",הגדרות!$B$4,IF(D8="EUR",הגדרות!$B$5,1)))</f>
         <v>37</v>
       </c>
-      <c r="L8" s="17" t="n">
+      <c r="L8" s="18" t="n">
         <f aca="false">IF(C8="","",IF(OR(E8="חודשי",E8="לפי שימוש"),K8,IF(E8="שנתי",K8/12,0)))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="D9" s="15" t="s">
+      <c r="C9" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="D9" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="G9" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="H9" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="I9" s="15" t="s">
+      <c r="H9" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="I9" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="J9" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="K9" s="17" t="n">
+      <c r="J9" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="K9" s="18" t="n">
         <f aca="false">IF(C9="","",C9*IF(D9="USD",הגדרות!$B$4,IF(D9="EUR",הגדרות!$B$5,1)))</f>
-        <v>55.5</v>
-      </c>
-      <c r="L9" s="17" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="L9" s="18" t="n">
         <f aca="false">IF(C9="","",IF(OR(E9="חודשי",E9="לפי שימוש"),K9,IF(E9="שנתי",K9/12,0)))</f>
-        <v>55.5</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B10" s="15" t="s">
+        <v>40.7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="17" t="n">
         <v>49</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="E10" s="15" t="s">
+      <c r="D10" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E10" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="G10" s="15" t="s">
+      <c r="F10" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="G10" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15" t="s">
+      <c r="H10" s="16"/>
+      <c r="I10" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="J10" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="K10" s="17" t="n">
+      <c r="J10" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="K10" s="18" t="n">
         <f aca="false">IF(C10="","",C10*IF(D10="USD",הגדרות!$B$4,IF(D10="EUR",הגדרות!$B$5,1)))</f>
         <v>196</v>
       </c>
-      <c r="L10" s="17" t="n">
+      <c r="L10" s="18" t="n">
         <f aca="false">IF(C10="","",IF(OR(E10="חודשי",E10="לפי שימוש"),K10,IF(E10="שנתי",K10/12,0)))</f>
         <v>196</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="B11" s="15" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="16" t="n">
+      <c r="C11" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="F11" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="G11" s="15" t="s">
+      <c r="F11" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15" t="s">
+      <c r="H11" s="16"/>
+      <c r="I11" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="J11" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="K11" s="17" t="n">
+      <c r="J11" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="K11" s="18" t="n">
         <f aca="false">IF(C11="","",C11*IF(D11="USD",הגדרות!$B$4,IF(D11="EUR",הגדרות!$B$5,1)))</f>
         <v>10</v>
       </c>
-      <c r="L11" s="17" t="n">
+      <c r="L11" s="18" t="n">
         <f aca="false">IF(C11="","",IF(OR(E11="חודשי",E11="לפי שימוש"),K11,IF(E11="שנתי",K11/12,0)))</f>
         <v>10</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="17" t="str">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="18" t="str">
         <f aca="false">IF(C12="","",C12*IF(D12="USD",הגדרות!$B$4,IF(D12="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L12" s="17" t="str">
+      <c r="L12" s="18" t="str">
         <f aca="false">IF(C12="","",IF(OR(E12="חודשי",E12="לפי שימוש"),K12,IF(E12="שנתי",K12/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="17" t="str">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="15"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="18" t="str">
         <f aca="false">IF(C13="","",C13*IF(D13="USD",הגדרות!$B$4,IF(D13="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L13" s="17" t="str">
+      <c r="L13" s="18" t="str">
         <f aca="false">IF(C13="","",IF(OR(E13="חודשי",E13="לפי שימוש"),K13,IF(E13="שנתי",K13/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="17" t="str">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="15"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="18" t="str">
         <f aca="false">IF(C14="","",C14*IF(D14="USD",הגדרות!$B$4,IF(D14="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L14" s="17" t="str">
+      <c r="L14" s="18" t="str">
         <f aca="false">IF(C14="","",IF(OR(E14="חודשי",E14="לפי שימוש"),K14,IF(E14="שנתי",K14/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="17" t="str">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="18" t="str">
         <f aca="false">IF(C15="","",C15*IF(D15="USD",הגדרות!$B$4,IF(D15="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L15" s="17" t="str">
+      <c r="L15" s="18" t="str">
         <f aca="false">IF(C15="","",IF(OR(E15="חודשי",E15="לפי שימוש"),K15,IF(E15="שנתי",K15/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="17" t="str">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="15"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="18" t="str">
         <f aca="false">IF(C16="","",C16*IF(D16="USD",הגדרות!$B$4,IF(D16="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L16" s="17" t="str">
+      <c r="L16" s="18" t="str">
         <f aca="false">IF(C16="","",IF(OR(E16="חודשי",E16="לפי שימוש"),K16,IF(E16="שנתי",K16/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="17" t="str">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="15"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="18" t="str">
         <f aca="false">IF(C17="","",C17*IF(D17="USD",הגדרות!$B$4,IF(D17="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L17" s="17" t="str">
+      <c r="L17" s="18" t="str">
         <f aca="false">IF(C17="","",IF(OR(E17="חודשי",E17="לפי שימוש"),K17,IF(E17="שנתי",K17/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="17" t="str">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="15"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="18" t="str">
         <f aca="false">IF(C18="","",C18*IF(D18="USD",הגדרות!$B$4,IF(D18="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L18" s="17" t="str">
+      <c r="L18" s="18" t="str">
         <f aca="false">IF(C18="","",IF(OR(E18="חודשי",E18="לפי שימוש"),K18,IF(E18="שנתי",K18/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14"/>
-      <c r="B19" s="15"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="17" t="str">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="15"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="18" t="str">
         <f aca="false">IF(C19="","",C19*IF(D19="USD",הגדרות!$B$4,IF(D19="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L19" s="17" t="str">
+      <c r="L19" s="18" t="str">
         <f aca="false">IF(C19="","",IF(OR(E19="חודשי",E19="לפי שימוש"),K19,IF(E19="שנתי",K19/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="17" t="str">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="18" t="str">
         <f aca="false">IF(C20="","",C20*IF(D20="USD",הגדרות!$B$4,IF(D20="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L20" s="17" t="str">
+      <c r="L20" s="18" t="str">
         <f aca="false">IF(C20="","",IF(OR(E20="חודשי",E20="לפי שימוש"),K20,IF(E20="שנתי",K20/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14"/>
-      <c r="B21" s="15"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="17" t="str">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="18" t="str">
         <f aca="false">IF(C21="","",C21*IF(D21="USD",הגדרות!$B$4,IF(D21="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L21" s="17" t="str">
+      <c r="L21" s="18" t="str">
         <f aca="false">IF(C21="","",IF(OR(E21="חודשי",E21="לפי שימוש"),K21,IF(E21="שנתי",K21/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="17" t="str">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="18" t="str">
         <f aca="false">IF(C22="","",C22*IF(D22="USD",הגדרות!$B$4,IF(D22="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L22" s="17" t="str">
+      <c r="L22" s="18" t="str">
         <f aca="false">IF(C22="","",IF(OR(E22="חודשי",E22="לפי שימוש"),K22,IF(E22="שנתי",K22/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14"/>
-      <c r="B23" s="15"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="17" t="str">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="18" t="str">
         <f aca="false">IF(C23="","",C23*IF(D23="USD",הגדרות!$B$4,IF(D23="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L23" s="17" t="str">
+      <c r="L23" s="18" t="str">
         <f aca="false">IF(C23="","",IF(OR(E23="חודשי",E23="לפי שימוש"),K23,IF(E23="שנתי",K23/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="17" t="str">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="16"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="18" t="str">
         <f aca="false">IF(C24="","",C24*IF(D24="USD",הגדרות!$B$4,IF(D24="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L24" s="17" t="str">
+      <c r="L24" s="18" t="str">
         <f aca="false">IF(C24="","",IF(OR(E24="חודשי",E24="לפי שימוש"),K24,IF(E24="שנתי",K24/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14"/>
-      <c r="B25" s="15"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="17" t="str">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="15"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="18" t="str">
         <f aca="false">IF(C25="","",C25*IF(D25="USD",הגדרות!$B$4,IF(D25="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L25" s="17" t="str">
+      <c r="L25" s="18" t="str">
         <f aca="false">IF(C25="","",IF(OR(E25="חודשי",E25="לפי שימוש"),K25,IF(E25="שנתי",K25/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="17" t="str">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="18" t="str">
         <f aca="false">IF(C26="","",C26*IF(D26="USD",הגדרות!$B$4,IF(D26="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L26" s="17" t="str">
+      <c r="L26" s="18" t="str">
         <f aca="false">IF(C26="","",IF(OR(E26="חודשי",E26="לפי שימוש"),K26,IF(E26="שנתי",K26/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="15"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="17" t="str">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="15"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="15"/>
+      <c r="K27" s="18" t="str">
         <f aca="false">IF(C27="","",C27*IF(D27="USD",הגדרות!$B$4,IF(D27="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L27" s="17" t="str">
+      <c r="L27" s="18" t="str">
         <f aca="false">IF(C27="","",IF(OR(E27="חודשי",E27="לפי שימוש"),K27,IF(E27="שנתי",K27/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14"/>
-      <c r="B28" s="15"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="14"/>
-      <c r="K28" s="17" t="str">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="15"/>
+      <c r="K28" s="18" t="str">
         <f aca="false">IF(C28="","",C28*IF(D28="USD",הגדרות!$B$4,IF(D28="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L28" s="17" t="str">
+      <c r="L28" s="18" t="str">
         <f aca="false">IF(C28="","",IF(OR(E28="חודשי",E28="לפי שימוש"),K28,IF(E28="שנתי",K28/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14"/>
-      <c r="B29" s="15"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="14"/>
-      <c r="K29" s="17" t="str">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="18" t="str">
         <f aca="false">IF(C29="","",C29*IF(D29="USD",הגדרות!$B$4,IF(D29="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L29" s="17" t="str">
+      <c r="L29" s="18" t="str">
         <f aca="false">IF(C29="","",IF(OR(E29="חודשי",E29="לפי שימוש"),K29,IF(E29="שנתי",K29/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14"/>
-      <c r="B30" s="15"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="15"/>
-      <c r="I30" s="15"/>
-      <c r="J30" s="14"/>
-      <c r="K30" s="17" t="str">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="16"/>
+      <c r="I30" s="16"/>
+      <c r="J30" s="15"/>
+      <c r="K30" s="18" t="str">
         <f aca="false">IF(C30="","",C30*IF(D30="USD",הגדרות!$B$4,IF(D30="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L30" s="17" t="str">
+      <c r="L30" s="18" t="str">
         <f aca="false">IF(C30="","",IF(OR(E30="חודשי",E30="לפי שימוש"),K30,IF(E30="שנתי",K30/12,0)))</f>
         <v/>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14"/>
-      <c r="B31" s="15"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="17" t="str">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="15"/>
+      <c r="K31" s="18" t="str">
         <f aca="false">IF(C31="","",C31*IF(D31="USD",הגדרות!$B$4,IF(D31="EUR",הגדרות!$B$5,1)))</f>
         <v/>
       </c>
-      <c r="L31" s="17" t="str">
+      <c r="L31" s="18" t="str">
         <f aca="false">IF(C31="","",IF(OR(E31="חודשי",E31="לפי שימוש"),K31,IF(E31="שנתי",K31/12,0)))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
UltraMsg subscription ended and is not renewed; Anthropic monthly cap set
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASRMwiCmV7VLN1LwrbbDK1
</commit_message>
<xml_diff>
--- a/automation-agency/expenses.xlsx
+++ b/automation-agency/expenses.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
   <si>
     <t xml:space="preserve">🔑 חנן המנעולן: כמה נכנס, כמה יוצא, ועל מי</t>
   </si>
@@ -112,7 +112,10 @@
     <t xml:space="preserve">UltraMsg (מספר הבדיקות)</t>
   </si>
   <si>
-    <t xml:space="preserve">39 דולר. אפשר לבטל אחרי שחנן עובר ל-360dialog</t>
+    <t xml:space="preserve">בוטל</t>
+  </si>
+  <si>
+    <t xml:space="preserve">המנוי פג ב-16/10/2026. לבדיקות עוברים ל-Dualhook על המספר של השותף</t>
   </si>
   <si>
     <t xml:space="preserve">360dialog (החיבור הרשמי למספר של חנן)</t>
@@ -470,8 +473,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -923,446 +930,446 @@
   <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>1000</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="9" t="n">
         <v>46305</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="9" t="s">
+      <c r="E6" s="8"/>
+      <c r="F6" s="10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="9" t="s">
+      <c r="D7" s="9"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="9" t="s">
+      <c r="D8" s="9"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="10" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <v>18.5</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="7" t="s">
+      <c r="C12" s="13"/>
+      <c r="D12" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="13" t="n">
         <v>40.7</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="13" t="n">
         <v>37</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="13" t="n">
         <v>144.3</v>
       </c>
-      <c r="C14" s="12"/>
-      <c r="D14" s="7" t="s">
+      <c r="C14" s="13"/>
+      <c r="D14" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>196</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" s="13"/>
+      <c r="D16" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="13"/>
+      <c r="D17" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="12" t="n">
-        <v>196</v>
-      </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="12"/>
-      <c r="D17" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="13"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="13"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="13"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+      <c r="F17" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="15" t="n">
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="14"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="14"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="16" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
-        <v>409.5</v>
-      </c>
-      <c r="C21" s="15" t="n">
+        <v>265.2</v>
+      </c>
+      <c r="C21" s="16" t="n">
         <f aca="false">SUMIFS(C12:C20,D12:D20,"&lt;&gt;בוטל")</f>
         <v>37</v>
       </c>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-    </row>
-    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="18" t="s">
+      <c r="A23" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+    </row>
+    <row r="24" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="19" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+      <c r="C24" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B25" s="20" t="n">
+    </row>
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="21" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="C25" s="20" t="n">
+      <c r="C25" s="21" t="n">
         <f aca="false">B8</f>
         <v>500</v>
       </c>
-      <c r="D25" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-    </row>
-    <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="s">
+      <c r="D25" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="22" t="n">
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+    </row>
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"עכשיו")</f>
-        <v>203.5</v>
-      </c>
-      <c r="C26" s="22" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="C26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
-        <v>409.5</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27" s="23" t="n">
+        <v>265.2</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="24" t="n">
         <f aca="false">B25-B26</f>
-        <v>-203.5</v>
-      </c>
-      <c r="C27" s="23" t="n">
+        <v>-59.2</v>
+      </c>
+      <c r="C27" s="24" t="n">
         <f aca="false">C25-C26</f>
-        <v>90.5</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="24" t="n">
+        <v>234.8</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="25" t="n">
         <f aca="false">SUMIFS(B6:B7,C6:C7,"כן")</f>
         <v>1000</v>
       </c>
-      <c r="C28" s="25" t="n">
+      <c r="C28" s="26" t="n">
         <f aca="false">SUMIFS(B6:B7,C6:C7,"לא")</f>
         <v>1500</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="C31" s="27" t="s">
+      <c r="A30" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="28" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B32" s="28" t="n">
+      <c r="A32" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="29" t="n">
         <v>0.5</v>
       </c>
-      <c r="C32" s="29" t="n">
+      <c r="C32" s="30" t="n">
         <f aca="false">1-B32</f>
         <v>0.5</v>
       </c>
-      <c r="D32" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="s">
+      <c r="D32" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="30" t="n">
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="31" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"אריאל")+SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"חצי חצי")/2</f>
         <v>0</v>
       </c>
-      <c r="C33" s="30" t="n">
+      <c r="C33" s="31" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"השותף")+SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"חצי חצי")/2</f>
-        <v>409.5</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="B34" s="31" t="n">
+        <v>265.2</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="B34" s="32" t="n">
         <f aca="false">C27*B32</f>
-        <v>45.25</v>
-      </c>
-      <c r="C34" s="31" t="n">
+        <v>117.4</v>
+      </c>
+      <c r="C34" s="32" t="n">
         <f aca="false">C27*C32</f>
-        <v>45.25</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="32" t="s">
-        <v>53</v>
-      </c>
-      <c r="B35" s="33" t="n">
+        <v>117.4</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B35" s="34" t="n">
         <f aca="false">B33+B34</f>
-        <v>45.25</v>
-      </c>
-      <c r="C35" s="33" t="n">
+        <v>117.4</v>
+      </c>
+      <c r="C35" s="34" t="n">
         <f aca="false">C33+C34</f>
-        <v>454.75</v>
-      </c>
-      <c r="D35" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
+        <v>382.6</v>
+      </c>
+      <c r="D35" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
Money sheet: Dualhook instead of 360dialog, Anthropic on Haiku
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASRMwiCmV7VLN1LwrbbDK1
</commit_message>
<xml_diff>
--- a/automation-agency/expenses.xlsx
+++ b/automation-agency/expenses.xlsx
@@ -106,7 +106,7 @@
     <t xml:space="preserve">Anthropic (המוח של הבוט)</t>
   </si>
   <si>
-    <t xml:space="preserve">בערך 11 דולר בחודש. "פעם אחת" = הטעינה הראשונה, 10 דולר</t>
+    <t xml:space="preserve">מ-20/10 על Haiku: הערכה, פחות מ-1.5 דולר בחודש (על Opus היה בערך 11). "פעם אחת" = הטעינה הראשונה, 10 דולר</t>
   </si>
   <si>
     <t xml:space="preserve">UltraMsg (מספר הבדיקות)</t>
@@ -118,13 +118,13 @@
     <t xml:space="preserve">המנוי פג ב-16/10/2026. לבדיקות עוברים ל-Dualhook על המספר של השותף</t>
   </si>
   <si>
-    <t xml:space="preserve">360dialog (החיבור הרשמי למספר של חנן)</t>
+    <t xml:space="preserve">Dualhook (החיבור הרשמי למספר של חנן)</t>
   </si>
   <si>
     <t xml:space="preserve">מיום החיבור</t>
   </si>
   <si>
-    <t xml:space="preserve">49 יורו</t>
+    <t xml:space="preserve">12 דולר לחודש. לבדוק ב-Billing אם דולר או יורו (ביורו בערך 48)</t>
   </si>
   <si>
     <t xml:space="preserve">Meta (תזכורות וביקורות)</t>
@@ -1090,7 +1090,7 @@
         <v>27</v>
       </c>
       <c r="B13" s="13" t="n">
-        <v>40.7</v>
+        <v>5</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>37</v>
@@ -1128,7 +1128,7 @@
         <v>32</v>
       </c>
       <c r="B15" s="13" t="n">
-        <v>196</v>
+        <v>45</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="8" t="s">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B21" s="16" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
-        <v>265.2</v>
+        <v>78.5</v>
       </c>
       <c r="C21" s="16" t="n">
         <f aca="false">SUMIFS(C12:C20,D12:D20,"&lt;&gt;בוטל")</f>
@@ -1259,11 +1259,11 @@
       </c>
       <c r="B26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"עכשיו")</f>
-        <v>59.2</v>
+        <v>23.5</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
-        <v>265.2</v>
+        <v>78.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1272,11 +1272,11 @@
       </c>
       <c r="B27" s="24" t="n">
         <f aca="false">B25-B26</f>
-        <v>-59.2</v>
+        <v>-23.5</v>
       </c>
       <c r="C27" s="24" t="n">
         <f aca="false">C25-C26</f>
-        <v>234.8</v>
+        <v>421.5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"השותף")+SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"חצי חצי")/2</f>
-        <v>265.2</v>
+        <v>78.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1346,11 +1346,11 @@
       </c>
       <c r="B34" s="32" t="n">
         <f aca="false">C27*B32</f>
-        <v>117.4</v>
+        <v>210.75</v>
       </c>
       <c r="C34" s="32" t="n">
         <f aca="false">C27*C32</f>
-        <v>117.4</v>
+        <v>210.75</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1359,11 +1359,11 @@
       </c>
       <c r="B35" s="34" t="n">
         <f aca="false">B33+B34</f>
-        <v>117.4</v>
+        <v>210.75</v>
       </c>
       <c r="C35" s="34" t="n">
         <f aca="false">C33+C34</f>
-        <v>382.6</v>
+        <v>289.25</v>
       </c>
       <c r="D35" s="22" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Money sheet: Anthropic on Sonnet, Meta billed in dollars
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASRMwiCmV7VLN1LwrbbDK1
</commit_message>
<xml_diff>
--- a/automation-agency/expenses.xlsx
+++ b/automation-agency/expenses.xlsx
@@ -106,7 +106,7 @@
     <t xml:space="preserve">Anthropic (המוח של הבוט)</t>
   </si>
   <si>
-    <t xml:space="preserve">מ-20/10 על Haiku: הערכה, פחות מ-1.5 דולר בחודש (על Opus היה בערך 11). "פעם אחת" = הטעינה הראשונה, 10 דולר</t>
+    <t xml:space="preserve">מ-20/10 על Sonnet: הערכה, בערך 2-3 דולר בחודש (על Opus היה בערך 11). "פעם אחת" = הטעינה הראשונה, 10 דולר</t>
   </si>
   <si>
     <t xml:space="preserve">UltraMsg (מספר הבדיקות)</t>
@@ -130,7 +130,7 @@
     <t xml:space="preserve">Meta (תזכורות וביקורות)</t>
   </si>
   <si>
-    <t xml:space="preserve">הערכה, אגורות להודעה</t>
+    <t xml:space="preserve">הערכה, אגורות להודעה. החיוב בדולר (Meta לא מחייבת בשקלים)</t>
   </si>
   <si>
     <t xml:space="preserve">GitHub (הקוד)</t>
@@ -1090,7 +1090,7 @@
         <v>27</v>
       </c>
       <c r="B13" s="13" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>37</v>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="B21" s="16" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
-        <v>78.5</v>
+        <v>83.5</v>
       </c>
       <c r="C21" s="16" t="n">
         <f aca="false">SUMIFS(C12:C20,D12:D20,"&lt;&gt;בוטל")</f>
@@ -1259,11 +1259,11 @@
       </c>
       <c r="B26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"עכשיו")</f>
-        <v>23.5</v>
+        <v>28.5</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
-        <v>78.5</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1272,11 +1272,11 @@
       </c>
       <c r="B27" s="24" t="n">
         <f aca="false">B25-B26</f>
-        <v>-23.5</v>
+        <v>-28.5</v>
       </c>
       <c r="C27" s="24" t="n">
         <f aca="false">C25-C26</f>
-        <v>421.5</v>
+        <v>416.5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"השותף")+SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"חצי חצי")/2</f>
-        <v>78.5</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1346,11 +1346,11 @@
       </c>
       <c r="B34" s="32" t="n">
         <f aca="false">C27*B32</f>
-        <v>210.75</v>
+        <v>208.25</v>
       </c>
       <c r="C34" s="32" t="n">
         <f aca="false">C27*C32</f>
-        <v>210.75</v>
+        <v>208.25</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1359,11 +1359,11 @@
       </c>
       <c r="B35" s="34" t="n">
         <f aca="false">B33+B34</f>
-        <v>210.75</v>
+        <v>208.25</v>
       </c>
       <c r="C35" s="34" t="n">
         <f aca="false">C33+C34</f>
-        <v>289.25</v>
+        <v>291.75</v>
       </c>
       <c r="D35" s="22" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Money sheet: UltraMsg row removed; Dualhook and Meta active from today
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASRMwiCmV7VLN1LwrbbDK1
</commit_message>
<xml_diff>
--- a/automation-agency/expenses.xlsx
+++ b/automation-agency/expenses.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="52">
   <si>
     <t xml:space="preserve">🔑 חנן המנעולן: כמה נכנס, כמה יוצא, ועל מי</t>
   </si>
@@ -109,19 +109,7 @@
     <t xml:space="preserve">מ-20/10 על Sonnet: הערכה, בערך 2-3 דולר בחודש (על Opus היה בערך 11). "פעם אחת" = הטעינה הראשונה, 10 דולר</t>
   </si>
   <si>
-    <t xml:space="preserve">UltraMsg (מספר הבדיקות)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">בוטל</t>
-  </si>
-  <si>
-    <t xml:space="preserve">המנוי פג ב-16/10/2026. לבדיקות עוברים ל-Dualhook על המספר של השותף</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dualhook (החיבור הרשמי למספר של חנן)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">מיום החיבור</t>
   </si>
   <si>
     <t xml:space="preserve">12 דולר לחודש. לבדוק ב-Billing אם דולר או יורו (ביורו בערך 48)</t>
@@ -1110,72 +1098,62 @@
         <v>29</v>
       </c>
       <c r="B14" s="13" t="n">
-        <v>144.3</v>
+        <v>45</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="8" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>25</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" s="13" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="8" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>25</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B16" s="13" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="8" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="A17" s="6"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>39</v>
-      </c>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6"/>
@@ -1203,7 +1181,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B21" s="16" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
@@ -1219,7 +1197,7 @@
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -1229,15 +1207,15 @@
     </row>
     <row r="24" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="19" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B25" s="21" t="n">
         <f aca="false">0</f>
@@ -1248,18 +1226,18 @@
         <v>500</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E25" s="22"/>
       <c r="F25" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"עכשיו")</f>
-        <v>28.5</v>
+        <v>83.5</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
@@ -1268,11 +1246,11 @@
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B27" s="24" t="n">
         <f aca="false">B25-B26</f>
-        <v>-28.5</v>
+        <v>-83.5</v>
       </c>
       <c r="C27" s="24" t="n">
         <f aca="false">C25-C26</f>
@@ -1281,7 +1259,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B28" s="25" t="n">
         <f aca="false">SUMIFS(B6:B7,C6:C7,"כן")</f>
@@ -1294,7 +1272,7 @@
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="27" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
@@ -1304,7 +1282,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="28" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C31" s="28" t="s">
         <v>25</v>
@@ -1312,7 +1290,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B32" s="29" t="n">
         <v>0.5</v>
@@ -1322,14 +1300,14 @@
         <v>0.5</v>
       </c>
       <c r="D32" s="22" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E32" s="22"/>
       <c r="F32" s="22"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B33" s="31" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"אריאל")+SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"חצי חצי")/2</f>
@@ -1342,7 +1320,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B34" s="32" t="n">
         <f aca="false">C27*B32</f>
@@ -1355,7 +1333,7 @@
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="33" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B35" s="34" t="n">
         <f aca="false">B33+B34</f>
@@ -1366,7 +1344,7 @@
         <v>291.75</v>
       </c>
       <c r="D35" s="22" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E35" s="22"/>
       <c r="F35" s="22"/>

</xml_diff>

<commit_message>
Money sheet: domain onerishon.com added (yearly, per month), notes corrected (Anthropic on Sonnet, Dualhook 12 not 49 euro, Meta)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASRMwiCmV7VLN1LwrbbDK1
</commit_message>
<xml_diff>
--- a/automation-agency/expenses.xlsx
+++ b/automation-agency/expenses.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="54">
   <si>
     <t xml:space="preserve">🔑 חנן המנעולן: כמה נכנס, כמה יוצא, ועל מי</t>
   </si>
@@ -100,25 +100,25 @@
     <t xml:space="preserve">השותף</t>
   </si>
   <si>
-    <t xml:space="preserve">5 דולר</t>
+    <t xml:space="preserve">5 דולר לחודש</t>
   </si>
   <si>
     <t xml:space="preserve">Anthropic (המוח של הבוט)</t>
   </si>
   <si>
-    <t xml:space="preserve">מ-20/10 על Sonnet: הערכה, בערך 2-3 דולר בחודש (על Opus היה בערך 11). "פעם אחת" = הטעינה הראשונה, 10 דולר</t>
+    <t xml:space="preserve">מ-21/10 על Sonnet: הערכה 2-3 דולר בחודש (על Opus היה בערך 11). "פעם אחת" = הטעינה הראשונה, 10 דולר</t>
   </si>
   <si>
     <t xml:space="preserve">Dualhook (החיבור הרשמי למספר של חנן)</t>
   </si>
   <si>
-    <t xml:space="preserve">12 דולר לחודש. לבדוק ב-Billing אם דולר או יורו (ביורו בערך 48)</t>
+    <t xml:space="preserve">12 בחודש למספר של חנן. לבדוק ב-Billing אם דולר (בערך 42 ₪) או יורו (בערך 48 ₪). לא 49 יורו: זה היה המחיר של 360dialog שלא לקחנו</t>
   </si>
   <si>
     <t xml:space="preserve">Meta (תזכורות וביקורות)</t>
   </si>
   <si>
-    <t xml:space="preserve">הערכה, אגורות להודעה. החיוב בדולר (Meta לא מחייבת בשקלים)</t>
+    <t xml:space="preserve">הערכה, אגורות להודעה, רק על הודעות ללקוח שלא כתב ב-24 שעות. החיוב בדולר</t>
   </si>
   <si>
     <t xml:space="preserve">GitHub (הקוד)</t>
@@ -128,6 +128,12 @@
   </si>
   <si>
     <t xml:space="preserve">חינם</t>
+  </si>
+  <si>
+    <t xml:space="preserve">דומיין onerishon.com (הכתובת לכפתורים במייל)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.46 דולר לשנה, חידוש אוטומטי דלוק. "בחודש" = השנתי חלקי 12. "פעם אחת" = התשלום השנתי</t>
   </si>
   <si>
     <t xml:space="preserve">סה"כ</t>
@@ -1148,12 +1154,24 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="10"/>
+      <c r="A17" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>38</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6"/>
@@ -1181,15 +1199,15 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B21" s="16" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
-        <v>83.5</v>
+        <v>86.5</v>
       </c>
       <c r="C21" s="16" t="n">
         <f aca="false">SUMIFS(C12:C20,D12:D20,"&lt;&gt;בוטל")</f>
-        <v>37</v>
+        <v>75</v>
       </c>
       <c r="D21" s="17"/>
       <c r="E21" s="17"/>
@@ -1197,7 +1215,7 @@
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -1207,15 +1225,15 @@
     </row>
     <row r="24" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="19" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B25" s="21" t="n">
         <f aca="false">0</f>
@@ -1226,40 +1244,40 @@
         <v>500</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E25" s="22"/>
       <c r="F25" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"עכשיו")</f>
-        <v>83.5</v>
+        <v>86.5</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל")</f>
-        <v>83.5</v>
+        <v>86.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B27" s="24" t="n">
         <f aca="false">B25-B26</f>
-        <v>-83.5</v>
+        <v>-86.5</v>
       </c>
       <c r="C27" s="24" t="n">
         <f aca="false">C25-C26</f>
-        <v>416.5</v>
+        <v>413.5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B28" s="25" t="n">
         <f aca="false">SUMIFS(B6:B7,C6:C7,"כן")</f>
@@ -1272,7 +1290,7 @@
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="27" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
@@ -1290,7 +1308,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B32" s="29" t="n">
         <v>0.5</v>
@@ -1300,14 +1318,14 @@
         <v>0.5</v>
       </c>
       <c r="D32" s="22" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E32" s="22"/>
       <c r="F32" s="22"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B33" s="31" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"אריאל")+SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"חצי חצי")/2</f>
@@ -1315,36 +1333,36 @@
       </c>
       <c r="C33" s="31" t="n">
         <f aca="false">SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"השותף")+SUMIFS(B12:B20,D12:D20,"&lt;&gt;בוטל",E12:E20,"חצי חצי")/2</f>
-        <v>83.5</v>
+        <v>86.5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B34" s="32" t="n">
         <f aca="false">C27*B32</f>
-        <v>208.25</v>
+        <v>206.75</v>
       </c>
       <c r="C34" s="32" t="n">
         <f aca="false">C27*C32</f>
-        <v>208.25</v>
+        <v>206.75</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="33" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B35" s="34" t="n">
         <f aca="false">B33+B34</f>
-        <v>208.25</v>
+        <v>206.75</v>
       </c>
       <c r="C35" s="34" t="n">
         <f aca="false">C33+C34</f>
-        <v>291.75</v>
+        <v>293.25</v>
       </c>
       <c r="D35" s="22" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E35" s="22"/>
       <c r="F35" s="22"/>

</xml_diff>